<commit_message>
Update state and Excel log
</commit_message>
<xml_diff>
--- a/vr_portfolio_log.xlsx
+++ b/vr_portfolio_log.xlsx
@@ -49,7 +49,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +66,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
         <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -128,6 +134,9 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -771,26 +780,26 @@
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="B4" s="3" t="n">
-        <v>18383.37</v>
+        <v>20334.6</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>14402.24</v>
+        <v>18423.45</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>3981.13</v>
+        <v>1911.15</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>18423.45</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>15057.2504</v>
+        <v>14891.652</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>23526.95375</v>
+        <v>23268.20625</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>HOLD</t>
         </is>
       </c>
     </row>
@@ -894,19 +903,19 @@
         <v>200</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>14402.24</v>
+        <v>18423.45</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>3981.13</v>
+        <v>1911.15</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>18383.37</v>
+        <v>20334.6</v>
       </c>
       <c r="H8" s="6" t="n">
         <v>18423.45</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>0.2161</v>
+        <v>0.1037</v>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
@@ -914,24 +923,24 @@
         </is>
       </c>
       <c r="K8" s="8" t="n">
-        <v>0.0216</v>
+        <v>0.0104</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>18821.56</v>
+        <v>18614.57</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>15057.25</v>
+        <v>14891.65</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>23526.95</v>
-      </c>
-      <c r="O8" s="9" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>23268.21</v>
+      </c>
+      <c r="O8" s="14" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="P8" s="6" t="n">
-        <v>3981.13</v>
+        <v>191.12</v>
       </c>
     </row>
     <row r="9"/>
@@ -995,10 +1004,10 @@
         <v>1</v>
       </c>
       <c r="B13" s="12" t="n">
-        <v>71.84</v>
+        <v>71.22</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>71.84</v>
+        <v>71.22</v>
       </c>
       <c r="D13" s="13" t="n">
         <v>1</v>
@@ -1007,10 +1016,10 @@
         <v>1</v>
       </c>
       <c r="J13" s="12" t="n">
-        <v>73.41</v>
+        <v>72.31</v>
       </c>
       <c r="K13" s="12" t="n">
-        <v>440.45</v>
+        <v>433.85</v>
       </c>
       <c r="L13" s="13" t="n">
         <v>6</v>
@@ -1021,10 +1030,10 @@
         <v>2</v>
       </c>
       <c r="B14" s="12" t="n">
-        <v>71.79000000000001</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>71.79000000000001</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="D14" s="13" t="n">
         <v>1</v>
@@ -1033,10 +1042,10 @@
         <v>2</v>
       </c>
       <c r="J14" s="12" t="n">
-        <v>74.93000000000001</v>
+        <v>72.94</v>
       </c>
       <c r="K14" s="12" t="n">
-        <v>449.56</v>
+        <v>437.62</v>
       </c>
       <c r="L14" s="13" t="n">
         <v>6</v>
@@ -1047,10 +1056,10 @@
         <v>3</v>
       </c>
       <c r="B15" s="12" t="n">
-        <v>71.73999999999999</v>
+        <v>70.31</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>71.73999999999999</v>
+        <v>70.31</v>
       </c>
       <c r="D15" s="13" t="n">
         <v>1</v>
@@ -1059,10 +1068,10 @@
         <v>3</v>
       </c>
       <c r="J15" s="12" t="n">
-        <v>76.44</v>
+        <v>73.56</v>
       </c>
       <c r="K15" s="12" t="n">
-        <v>458.67</v>
+        <v>441.39</v>
       </c>
       <c r="L15" s="13" t="n">
         <v>6</v>
@@ -1073,10 +1082,10 @@
         <v>4</v>
       </c>
       <c r="B16" s="12" t="n">
-        <v>71.69</v>
+        <v>69.84999999999999</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>71.69</v>
+        <v>69.84999999999999</v>
       </c>
       <c r="D16" s="13" t="n">
         <v>1</v>
@@ -1085,10 +1094,10 @@
         <v>4</v>
       </c>
       <c r="J16" s="12" t="n">
-        <v>77.95999999999999</v>
+        <v>74.19</v>
       </c>
       <c r="K16" s="12" t="n">
-        <v>467.78</v>
+        <v>445.16</v>
       </c>
       <c r="L16" s="13" t="n">
         <v>6</v>
@@ -1099,10 +1108,10 @@
         <v>5</v>
       </c>
       <c r="B17" s="12" t="n">
-        <v>71.64</v>
+        <v>69.39</v>
       </c>
       <c r="C17" s="12" t="n">
-        <v>71.64</v>
+        <v>69.39</v>
       </c>
       <c r="D17" s="13" t="n">
         <v>1</v>
@@ -1111,10 +1120,10 @@
         <v>5</v>
       </c>
       <c r="J17" s="12" t="n">
-        <v>79.48</v>
+        <v>74.81999999999999</v>
       </c>
       <c r="K17" s="12" t="n">
-        <v>476.89</v>
+        <v>448.93</v>
       </c>
       <c r="L17" s="13" t="n">
         <v>6</v>
@@ -1125,10 +1134,10 @@
         <v>6</v>
       </c>
       <c r="B18" s="12" t="n">
-        <v>71.59</v>
+        <v>68.93000000000001</v>
       </c>
       <c r="C18" s="12" t="n">
-        <v>71.59</v>
+        <v>68.93000000000001</v>
       </c>
       <c r="D18" s="13" t="n">
         <v>1</v>
@@ -1137,10 +1146,10 @@
         <v>6</v>
       </c>
       <c r="J18" s="12" t="n">
-        <v>81</v>
+        <v>75.45</v>
       </c>
       <c r="K18" s="12" t="n">
-        <v>486</v>
+        <v>452.7</v>
       </c>
       <c r="L18" s="13" t="n">
         <v>6</v>
@@ -1151,10 +1160,10 @@
         <v>7</v>
       </c>
       <c r="B19" s="12" t="n">
-        <v>71.54000000000001</v>
+        <v>68.47</v>
       </c>
       <c r="C19" s="12" t="n">
-        <v>71.54000000000001</v>
+        <v>68.47</v>
       </c>
       <c r="D19" s="13" t="n">
         <v>1</v>
@@ -1163,10 +1172,10 @@
         <v>7</v>
       </c>
       <c r="J19" s="12" t="n">
-        <v>82.52</v>
+        <v>76.08</v>
       </c>
       <c r="K19" s="12" t="n">
-        <v>495.11</v>
+        <v>456.47</v>
       </c>
       <c r="L19" s="13" t="n">
         <v>6</v>
@@ -1177,10 +1186,10 @@
         <v>8</v>
       </c>
       <c r="B20" s="12" t="n">
-        <v>71.48999999999999</v>
+        <v>68.02</v>
       </c>
       <c r="C20" s="12" t="n">
-        <v>71.48999999999999</v>
+        <v>68.02</v>
       </c>
       <c r="D20" s="13" t="n">
         <v>1</v>
@@ -1189,10 +1198,10 @@
         <v>8</v>
       </c>
       <c r="J20" s="12" t="n">
-        <v>84.04000000000001</v>
+        <v>76.70999999999999</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>504.21</v>
+        <v>460.24</v>
       </c>
       <c r="L20" s="13" t="n">
         <v>6</v>
@@ -1203,10 +1212,10 @@
         <v>9</v>
       </c>
       <c r="B21" s="12" t="n">
-        <v>71.44</v>
+        <v>67.56</v>
       </c>
       <c r="C21" s="12" t="n">
-        <v>71.44</v>
+        <v>67.56</v>
       </c>
       <c r="D21" s="13" t="n">
         <v>1</v>
@@ -1215,10 +1224,10 @@
         <v>9</v>
       </c>
       <c r="J21" s="12" t="n">
-        <v>85.55</v>
+        <v>77.33</v>
       </c>
       <c r="K21" s="12" t="n">
-        <v>513.3200000000001</v>
+        <v>464.01</v>
       </c>
       <c r="L21" s="13" t="n">
         <v>6</v>
@@ -1229,10 +1238,10 @@
         <v>10</v>
       </c>
       <c r="B22" s="12" t="n">
-        <v>71.39</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="C22" s="12" t="n">
-        <v>71.39</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="D22" s="13" t="n">
         <v>1</v>
@@ -1241,10 +1250,10 @@
         <v>10</v>
       </c>
       <c r="J22" s="12" t="n">
-        <v>87.06999999999999</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="K22" s="12" t="n">
-        <v>522.4299999999999</v>
+        <v>467.78</v>
       </c>
       <c r="L22" s="13" t="n">
         <v>6</v>
@@ -1255,10 +1264,10 @@
         <v>11</v>
       </c>
       <c r="B23" s="12" t="n">
-        <v>71.34</v>
+        <v>66.64</v>
       </c>
       <c r="C23" s="12" t="n">
-        <v>71.34</v>
+        <v>66.64</v>
       </c>
       <c r="D23" s="13" t="n">
         <v>1</v>
@@ -1267,10 +1276,10 @@
         <v>11</v>
       </c>
       <c r="J23" s="12" t="n">
-        <v>88.59</v>
+        <v>78.59</v>
       </c>
       <c r="K23" s="12" t="n">
-        <v>531.54</v>
+        <v>471.55</v>
       </c>
       <c r="L23" s="13" t="n">
         <v>6</v>
@@ -1281,10 +1290,10 @@
         <v>12</v>
       </c>
       <c r="B24" s="12" t="n">
-        <v>71.29000000000001</v>
+        <v>66.18000000000001</v>
       </c>
       <c r="C24" s="12" t="n">
-        <v>71.29000000000001</v>
+        <v>66.18000000000001</v>
       </c>
       <c r="D24" s="13" t="n">
         <v>1</v>
@@ -1293,10 +1302,10 @@
         <v>12</v>
       </c>
       <c r="J24" s="12" t="n">
-        <v>90.11</v>
+        <v>79.22</v>
       </c>
       <c r="K24" s="12" t="n">
-        <v>540.65</v>
+        <v>475.32</v>
       </c>
       <c r="L24" s="13" t="n">
         <v>6</v>
@@ -1307,10 +1316,10 @@
         <v>13</v>
       </c>
       <c r="B25" s="12" t="n">
-        <v>71.23999999999999</v>
+        <v>65.73</v>
       </c>
       <c r="C25" s="12" t="n">
-        <v>71.23999999999999</v>
+        <v>65.73</v>
       </c>
       <c r="D25" s="13" t="n">
         <v>1</v>
@@ -1319,10 +1328,10 @@
         <v>13</v>
       </c>
       <c r="J25" s="12" t="n">
-        <v>91.63</v>
+        <v>79.84999999999999</v>
       </c>
       <c r="K25" s="12" t="n">
-        <v>549.76</v>
+        <v>479.09</v>
       </c>
       <c r="L25" s="13" t="n">
         <v>6</v>
@@ -1333,10 +1342,10 @@
         <v>14</v>
       </c>
       <c r="B26" s="12" t="n">
-        <v>71.19</v>
+        <v>65.27</v>
       </c>
       <c r="C26" s="12" t="n">
-        <v>71.19</v>
+        <v>65.27</v>
       </c>
       <c r="D26" s="13" t="n">
         <v>1</v>
@@ -1345,10 +1354,10 @@
         <v>14</v>
       </c>
       <c r="J26" s="12" t="n">
-        <v>93.15000000000001</v>
+        <v>80.48</v>
       </c>
       <c r="K26" s="12" t="n">
-        <v>558.87</v>
+        <v>482.86</v>
       </c>
       <c r="L26" s="13" t="n">
         <v>6</v>
@@ -1359,10 +1368,10 @@
         <v>15</v>
       </c>
       <c r="B27" s="12" t="n">
-        <v>71.14</v>
+        <v>64.81</v>
       </c>
       <c r="C27" s="12" t="n">
-        <v>71.14</v>
+        <v>64.81</v>
       </c>
       <c r="D27" s="13" t="n">
         <v>1</v>
@@ -1371,10 +1380,10 @@
         <v>15</v>
       </c>
       <c r="J27" s="12" t="n">
-        <v>94.66</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="K27" s="12" t="n">
-        <v>567.98</v>
+        <v>486.63</v>
       </c>
       <c r="L27" s="13" t="n">
         <v>6</v>
@@ -1385,10 +1394,10 @@
         <v>16</v>
       </c>
       <c r="B28" s="12" t="n">
-        <v>71.09</v>
+        <v>64.34999999999999</v>
       </c>
       <c r="C28" s="12" t="n">
-        <v>71.09</v>
+        <v>64.34999999999999</v>
       </c>
       <c r="D28" s="13" t="n">
         <v>1</v>
@@ -1397,10 +1406,10 @@
         <v>16</v>
       </c>
       <c r="J28" s="12" t="n">
-        <v>96.18000000000001</v>
+        <v>81.73</v>
       </c>
       <c r="K28" s="12" t="n">
-        <v>577.09</v>
+        <v>490.4</v>
       </c>
       <c r="L28" s="13" t="n">
         <v>6</v>
@@ -1411,10 +1420,10 @@
         <v>17</v>
       </c>
       <c r="B29" s="12" t="n">
-        <v>71.04000000000001</v>
+        <v>63.89</v>
       </c>
       <c r="C29" s="12" t="n">
-        <v>71.04000000000001</v>
+        <v>63.89</v>
       </c>
       <c r="D29" s="13" t="n">
         <v>1</v>
@@ -1423,10 +1432,10 @@
         <v>17</v>
       </c>
       <c r="J29" s="12" t="n">
-        <v>97.7</v>
+        <v>82.36</v>
       </c>
       <c r="K29" s="12" t="n">
-        <v>586.2</v>
+        <v>494.17</v>
       </c>
       <c r="L29" s="13" t="n">
         <v>6</v>
@@ -1437,10 +1446,10 @@
         <v>18</v>
       </c>
       <c r="B30" s="12" t="n">
-        <v>70.98999999999999</v>
+        <v>63.44</v>
       </c>
       <c r="C30" s="12" t="n">
-        <v>70.98999999999999</v>
+        <v>63.44</v>
       </c>
       <c r="D30" s="13" t="n">
         <v>1</v>
@@ -1449,10 +1458,10 @@
         <v>18</v>
       </c>
       <c r="J30" s="12" t="n">
-        <v>99.22</v>
+        <v>82.98999999999999</v>
       </c>
       <c r="K30" s="12" t="n">
-        <v>595.3099999999999</v>
+        <v>497.94</v>
       </c>
       <c r="L30" s="13" t="n">
         <v>6</v>
@@ -1463,10 +1472,10 @@
         <v>19</v>
       </c>
       <c r="B31" s="12" t="n">
-        <v>70.94</v>
+        <v>62.98</v>
       </c>
       <c r="C31" s="12" t="n">
-        <v>70.94</v>
+        <v>62.98</v>
       </c>
       <c r="D31" s="13" t="n">
         <v>1</v>
@@ -1475,10 +1484,10 @@
         <v>19</v>
       </c>
       <c r="J31" s="12" t="n">
-        <v>100.74</v>
+        <v>83.62</v>
       </c>
       <c r="K31" s="12" t="n">
-        <v>604.42</v>
+        <v>501.71</v>
       </c>
       <c r="L31" s="13" t="n">
         <v>6</v>
@@ -1489,10 +1498,10 @@
         <v>20</v>
       </c>
       <c r="B32" s="12" t="n">
-        <v>70.89</v>
+        <v>62.52</v>
       </c>
       <c r="C32" s="12" t="n">
-        <v>70.89</v>
+        <v>62.52</v>
       </c>
       <c r="D32" s="13" t="n">
         <v>1</v>
@@ -1501,10 +1510,10 @@
         <v>20</v>
       </c>
       <c r="J32" s="12" t="n">
-        <v>102.25</v>
+        <v>84.25</v>
       </c>
       <c r="K32" s="12" t="n">
-        <v>613.53</v>
+        <v>505.48</v>
       </c>
       <c r="L32" s="13" t="n">
         <v>6</v>
@@ -1515,10 +1524,10 @@
         <v>21</v>
       </c>
       <c r="B33" s="12" t="n">
-        <v>70.84</v>
+        <v>62.06</v>
       </c>
       <c r="C33" s="12" t="n">
-        <v>70.84</v>
+        <v>62.06</v>
       </c>
       <c r="D33" s="13" t="n">
         <v>1</v>
@@ -1527,10 +1536,10 @@
         <v>21</v>
       </c>
       <c r="J33" s="12" t="n">
-        <v>103.77</v>
+        <v>84.87</v>
       </c>
       <c r="K33" s="12" t="n">
-        <v>622.64</v>
+        <v>509.25</v>
       </c>
       <c r="L33" s="13" t="n">
         <v>6</v>
@@ -1541,10 +1550,10 @@
         <v>22</v>
       </c>
       <c r="B34" s="12" t="n">
-        <v>70.79000000000001</v>
+        <v>61.6</v>
       </c>
       <c r="C34" s="12" t="n">
-        <v>70.79000000000001</v>
+        <v>61.6</v>
       </c>
       <c r="D34" s="13" t="n">
         <v>1</v>
@@ -1553,10 +1562,10 @@
         <v>22</v>
       </c>
       <c r="J34" s="12" t="n">
-        <v>105.29</v>
+        <v>85.5</v>
       </c>
       <c r="K34" s="12" t="n">
-        <v>631.75</v>
+        <v>513.02</v>
       </c>
       <c r="L34" s="13" t="n">
         <v>6</v>
@@ -1567,10 +1576,10 @@
         <v>23</v>
       </c>
       <c r="B35" s="12" t="n">
-        <v>70.73999999999999</v>
+        <v>61.15</v>
       </c>
       <c r="C35" s="12" t="n">
-        <v>70.73999999999999</v>
+        <v>61.15</v>
       </c>
       <c r="D35" s="13" t="n">
         <v>1</v>
@@ -1579,10 +1588,10 @@
         <v>23</v>
       </c>
       <c r="J35" s="12" t="n">
-        <v>106.81</v>
+        <v>86.13</v>
       </c>
       <c r="K35" s="12" t="n">
-        <v>640.86</v>
+        <v>516.79</v>
       </c>
       <c r="L35" s="13" t="n">
         <v>6</v>
@@ -1593,10 +1602,10 @@
         <v>24</v>
       </c>
       <c r="B36" s="12" t="n">
-        <v>70.69</v>
+        <v>60.69</v>
       </c>
       <c r="C36" s="12" t="n">
-        <v>70.69</v>
+        <v>60.69</v>
       </c>
       <c r="D36" s="13" t="n">
         <v>1</v>
@@ -1605,10 +1614,10 @@
         <v>24</v>
       </c>
       <c r="J36" s="12" t="n">
-        <v>108.33</v>
+        <v>86.76000000000001</v>
       </c>
       <c r="K36" s="12" t="n">
-        <v>649.96</v>
+        <v>520.5599999999999</v>
       </c>
       <c r="L36" s="13" t="n">
         <v>6</v>
@@ -1619,10 +1628,10 @@
         <v>25</v>
       </c>
       <c r="B37" s="12" t="n">
-        <v>70.64</v>
+        <v>60.23</v>
       </c>
       <c r="C37" s="12" t="n">
-        <v>70.64</v>
+        <v>60.23</v>
       </c>
       <c r="D37" s="13" t="n">
         <v>1</v>
@@ -1631,10 +1640,10 @@
         <v>25</v>
       </c>
       <c r="J37" s="12" t="n">
-        <v>109.85</v>
+        <v>87.39</v>
       </c>
       <c r="K37" s="12" t="n">
-        <v>659.0700000000001</v>
+        <v>524.33</v>
       </c>
       <c r="L37" s="13" t="n">
         <v>6</v>
@@ -1645,10 +1654,10 @@
         <v>26</v>
       </c>
       <c r="B38" s="12" t="n">
-        <v>70.59</v>
+        <v>59.77</v>
       </c>
       <c r="C38" s="12" t="n">
-        <v>70.59</v>
+        <v>59.77</v>
       </c>
       <c r="D38" s="13" t="n">
         <v>1</v>
@@ -1657,10 +1666,10 @@
         <v>26</v>
       </c>
       <c r="J38" s="12" t="n">
-        <v>111.36</v>
+        <v>88.02</v>
       </c>
       <c r="K38" s="12" t="n">
-        <v>668.1799999999999</v>
+        <v>528.1</v>
       </c>
       <c r="L38" s="13" t="n">
         <v>6</v>
@@ -1671,10 +1680,10 @@
         <v>27</v>
       </c>
       <c r="B39" s="12" t="n">
-        <v>70.54000000000001</v>
+        <v>59.31</v>
       </c>
       <c r="C39" s="12" t="n">
-        <v>70.54000000000001</v>
+        <v>59.31</v>
       </c>
       <c r="D39" s="13" t="n">
         <v>1</v>
@@ -1683,10 +1692,10 @@
         <v>27</v>
       </c>
       <c r="J39" s="12" t="n">
-        <v>112.88</v>
+        <v>88.64</v>
       </c>
       <c r="K39" s="12" t="n">
-        <v>677.29</v>
+        <v>531.87</v>
       </c>
       <c r="L39" s="13" t="n">
         <v>6</v>
@@ -1697,10 +1706,10 @@
         <v>28</v>
       </c>
       <c r="B40" s="12" t="n">
-        <v>70.48999999999999</v>
+        <v>58.85</v>
       </c>
       <c r="C40" s="12" t="n">
-        <v>70.48999999999999</v>
+        <v>58.85</v>
       </c>
       <c r="D40" s="13" t="n">
         <v>1</v>
@@ -1709,10 +1718,10 @@
         <v>28</v>
       </c>
       <c r="J40" s="12" t="n">
-        <v>114.4</v>
+        <v>89.27</v>
       </c>
       <c r="K40" s="12" t="n">
-        <v>686.4</v>
+        <v>535.64</v>
       </c>
       <c r="L40" s="13" t="n">
         <v>6</v>
@@ -1723,10 +1732,10 @@
         <v>29</v>
       </c>
       <c r="B41" s="12" t="n">
-        <v>70.44</v>
+        <v>58.4</v>
       </c>
       <c r="C41" s="12" t="n">
-        <v>70.44</v>
+        <v>58.4</v>
       </c>
       <c r="D41" s="13" t="n">
         <v>1</v>
@@ -1735,10 +1744,10 @@
         <v>29</v>
       </c>
       <c r="J41" s="12" t="n">
-        <v>115.92</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="K41" s="12" t="n">
-        <v>695.51</v>
+        <v>539.41</v>
       </c>
       <c r="L41" s="13" t="n">
         <v>6</v>
@@ -1749,10 +1758,10 @@
         <v>30</v>
       </c>
       <c r="B42" s="12" t="n">
-        <v>70.39</v>
+        <v>57.94</v>
       </c>
       <c r="C42" s="12" t="n">
-        <v>70.39</v>
+        <v>57.94</v>
       </c>
       <c r="D42" s="13" t="n">
         <v>1</v>
@@ -1761,10 +1770,10 @@
         <v>30</v>
       </c>
       <c r="J42" s="12" t="n">
-        <v>117.44</v>
+        <v>90.53</v>
       </c>
       <c r="K42" s="12" t="n">
-        <v>704.62</v>
+        <v>543.1799999999999</v>
       </c>
       <c r="L42" s="13" t="n">
         <v>6</v>

</xml_diff>

<commit_message>
Switch VR 5.0 mode from deposit to lump_sum (거치식) with deposit_amount = 0
</commit_message>
<xml_diff>
--- a/vr_portfolio_log.xlsx
+++ b/vr_portfolio_log.xlsx
@@ -727,10 +727,10 @@
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
@@ -789,26 +789,26 @@
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="B4" s="3" t="n">
-        <v>19831.51</v>
+        <v>7170.37</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>14836</v>
+        <v>4058.27</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>4995.509999999998</v>
+        <v>3112.1</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>18423.45</v>
+        <v>4058.27</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>15138.4008</v>
+        <v>3714.058</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>23653.75125</v>
+        <v>5024.901999999999</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>HOLD</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>1회차 (6/14일)</t>
+          <t>2회차 (1/14일)</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1022,25 +1022,25 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>70.76000000000001</v>
+        <v>70.87</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>213</v>
+        <v>200</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>14836</v>
+        <v>4058.27</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>4995.51</v>
+        <v>3112.1</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>19831.51</v>
+        <v>7170.37</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>18423.45</v>
+        <v>4058.27</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>0.2711</v>
+        <v>0.7669</v>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
@@ -1048,24 +1048,24 @@
         </is>
       </c>
       <c r="K10" s="8" t="n">
-        <v>0.0271</v>
+        <v>0.0767</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>18923</v>
+        <v>4369.48</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>15138.4</v>
+        <v>3714.06</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>23653.75</v>
-      </c>
-      <c r="O10" s="9" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>5024.9</v>
+      </c>
+      <c r="O10" s="14" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="P10" s="6" t="n">
-        <v>4087</v>
+        <v>311.21</v>
       </c>
     </row>
     <row r="11">
@@ -1211,25 +1211,25 @@
         <v>1</v>
       </c>
       <c r="B15" s="12" t="n">
-        <v>69.48999999999999</v>
+        <v>71.48</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>138.98</v>
+        <v>71.48</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I15" s="11" t="n">
         <v>1</v>
       </c>
       <c r="J15" s="12" t="n">
-        <v>73.47</v>
+        <v>72.94</v>
       </c>
       <c r="K15" s="12" t="n">
-        <v>514.26</v>
+        <v>437.65</v>
       </c>
       <c r="L15" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
@@ -1237,25 +1237,25 @@
         <v>2</v>
       </c>
       <c r="B16" s="12" t="n">
-        <v>69.44</v>
+        <v>71.27</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>138.88</v>
+        <v>71.27</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I16" s="11" t="n">
         <v>2</v>
       </c>
       <c r="J16" s="12" t="n">
-        <v>74.75</v>
+        <v>73.48999999999999</v>
       </c>
       <c r="K16" s="12" t="n">
-        <v>523.28</v>
+        <v>440.92</v>
       </c>
       <c r="L16" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
@@ -1263,25 +1263,25 @@
         <v>3</v>
       </c>
       <c r="B17" s="12" t="n">
-        <v>69.39</v>
+        <v>71.06999999999999</v>
       </c>
       <c r="C17" s="12" t="n">
-        <v>138.78</v>
+        <v>71.06999999999999</v>
       </c>
       <c r="D17" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I17" s="11" t="n">
         <v>3</v>
       </c>
       <c r="J17" s="12" t="n">
-        <v>76.04000000000001</v>
+        <v>74.03</v>
       </c>
       <c r="K17" s="12" t="n">
-        <v>532.3099999999999</v>
+        <v>444.19</v>
       </c>
       <c r="L17" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -1289,25 +1289,25 @@
         <v>4</v>
       </c>
       <c r="B18" s="12" t="n">
-        <v>69.34</v>
+        <v>70.87</v>
       </c>
       <c r="C18" s="12" t="n">
-        <v>138.68</v>
+        <v>70.87</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I18" s="11" t="n">
         <v>4</v>
       </c>
       <c r="J18" s="12" t="n">
-        <v>77.33</v>
+        <v>74.58</v>
       </c>
       <c r="K18" s="12" t="n">
-        <v>541.34</v>
+        <v>447.47</v>
       </c>
       <c r="L18" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
@@ -1315,25 +1315,25 @@
         <v>5</v>
       </c>
       <c r="B19" s="12" t="n">
-        <v>69.29000000000001</v>
+        <v>70.67</v>
       </c>
       <c r="C19" s="12" t="n">
-        <v>138.58</v>
+        <v>70.67</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I19" s="11" t="n">
         <v>5</v>
       </c>
       <c r="J19" s="12" t="n">
-        <v>78.62</v>
+        <v>75.12</v>
       </c>
       <c r="K19" s="12" t="n">
-        <v>550.37</v>
+        <v>450.74</v>
       </c>
       <c r="L19" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -1341,25 +1341,25 @@
         <v>6</v>
       </c>
       <c r="B20" s="12" t="n">
-        <v>69.23999999999999</v>
+        <v>70.45999999999999</v>
       </c>
       <c r="C20" s="12" t="n">
-        <v>138.48</v>
+        <v>70.45999999999999</v>
       </c>
       <c r="D20" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I20" s="11" t="n">
         <v>6</v>
       </c>
       <c r="J20" s="12" t="n">
-        <v>79.91</v>
+        <v>75.67</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>559.4</v>
+        <v>454.01</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -1367,25 +1367,25 @@
         <v>7</v>
       </c>
       <c r="B21" s="12" t="n">
-        <v>69.19</v>
+        <v>70.26000000000001</v>
       </c>
       <c r="C21" s="12" t="n">
-        <v>138.38</v>
+        <v>70.26000000000001</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I21" s="11" t="n">
         <v>7</v>
       </c>
       <c r="J21" s="12" t="n">
-        <v>81.2</v>
+        <v>76.20999999999999</v>
       </c>
       <c r="K21" s="12" t="n">
-        <v>568.4299999999999</v>
+        <v>457.28</v>
       </c>
       <c r="L21" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
@@ -1393,25 +1393,25 @@
         <v>8</v>
       </c>
       <c r="B22" s="12" t="n">
-        <v>69.14</v>
+        <v>70.06</v>
       </c>
       <c r="C22" s="12" t="n">
-        <v>138.28</v>
+        <v>70.06</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I22" s="11" t="n">
         <v>8</v>
       </c>
       <c r="J22" s="12" t="n">
-        <v>82.48999999999999</v>
+        <v>76.76000000000001</v>
       </c>
       <c r="K22" s="12" t="n">
-        <v>577.46</v>
+        <v>460.55</v>
       </c>
       <c r="L22" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23">
@@ -1419,25 +1419,25 @@
         <v>9</v>
       </c>
       <c r="B23" s="12" t="n">
-        <v>69.09</v>
+        <v>69.86</v>
       </c>
       <c r="C23" s="12" t="n">
-        <v>138.18</v>
+        <v>69.86</v>
       </c>
       <c r="D23" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I23" s="11" t="n">
         <v>9</v>
       </c>
       <c r="J23" s="12" t="n">
-        <v>83.78</v>
+        <v>77.3</v>
       </c>
       <c r="K23" s="12" t="n">
-        <v>586.49</v>
+        <v>463.82</v>
       </c>
       <c r="L23" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
@@ -1445,25 +1445,25 @@
         <v>10</v>
       </c>
       <c r="B24" s="12" t="n">
-        <v>69.04000000000001</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="C24" s="12" t="n">
-        <v>138.08</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="D24" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I24" s="11" t="n">
         <v>10</v>
       </c>
       <c r="J24" s="12" t="n">
-        <v>85.06999999999999</v>
+        <v>77.84999999999999</v>
       </c>
       <c r="K24" s="12" t="n">
-        <v>595.52</v>
+        <v>467.09</v>
       </c>
       <c r="L24" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -1471,25 +1471,25 @@
         <v>11</v>
       </c>
       <c r="B25" s="12" t="n">
-        <v>68.98999999999999</v>
+        <v>69.45</v>
       </c>
       <c r="C25" s="12" t="n">
-        <v>137.98</v>
+        <v>69.45</v>
       </c>
       <c r="D25" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I25" s="11" t="n">
         <v>11</v>
       </c>
       <c r="J25" s="12" t="n">
-        <v>86.36</v>
+        <v>78.39</v>
       </c>
       <c r="K25" s="12" t="n">
-        <v>604.55</v>
+        <v>470.37</v>
       </c>
       <c r="L25" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -1497,25 +1497,25 @@
         <v>12</v>
       </c>
       <c r="B26" s="12" t="n">
-        <v>68.94</v>
+        <v>69.25</v>
       </c>
       <c r="C26" s="12" t="n">
-        <v>137.88</v>
+        <v>69.25</v>
       </c>
       <c r="D26" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I26" s="11" t="n">
         <v>12</v>
       </c>
       <c r="J26" s="12" t="n">
-        <v>87.65000000000001</v>
+        <v>78.94</v>
       </c>
       <c r="K26" s="12" t="n">
-        <v>613.5700000000001</v>
+        <v>473.64</v>
       </c>
       <c r="L26" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
@@ -1523,25 +1523,25 @@
         <v>13</v>
       </c>
       <c r="B27" s="12" t="n">
-        <v>68.89</v>
+        <v>69.05</v>
       </c>
       <c r="C27" s="12" t="n">
-        <v>137.78</v>
+        <v>69.05</v>
       </c>
       <c r="D27" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I27" s="11" t="n">
         <v>13</v>
       </c>
       <c r="J27" s="12" t="n">
-        <v>88.94</v>
+        <v>79.48</v>
       </c>
       <c r="K27" s="12" t="n">
-        <v>622.6</v>
+        <v>476.91</v>
       </c>
       <c r="L27" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28">
@@ -1552,22 +1552,22 @@
         <v>68.84</v>
       </c>
       <c r="C28" s="12" t="n">
-        <v>137.68</v>
+        <v>68.84</v>
       </c>
       <c r="D28" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I28" s="11" t="n">
         <v>14</v>
       </c>
       <c r="J28" s="12" t="n">
-        <v>90.23</v>
+        <v>80.03</v>
       </c>
       <c r="K28" s="12" t="n">
-        <v>631.63</v>
+        <v>480.18</v>
       </c>
       <c r="L28" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
@@ -1575,25 +1575,25 @@
         <v>15</v>
       </c>
       <c r="B29" s="12" t="n">
-        <v>68.79000000000001</v>
+        <v>68.64</v>
       </c>
       <c r="C29" s="12" t="n">
-        <v>137.58</v>
+        <v>68.64</v>
       </c>
       <c r="D29" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I29" s="11" t="n">
         <v>15</v>
       </c>
       <c r="J29" s="12" t="n">
-        <v>91.52</v>
+        <v>80.58</v>
       </c>
       <c r="K29" s="12" t="n">
-        <v>640.66</v>
+        <v>483.45</v>
       </c>
       <c r="L29" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
@@ -1601,25 +1601,25 @@
         <v>16</v>
       </c>
       <c r="B30" s="12" t="n">
-        <v>68.73999999999999</v>
+        <v>68.44</v>
       </c>
       <c r="C30" s="12" t="n">
-        <v>137.48</v>
+        <v>68.44</v>
       </c>
       <c r="D30" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I30" s="11" t="n">
         <v>16</v>
       </c>
       <c r="J30" s="12" t="n">
-        <v>92.81</v>
+        <v>81.12</v>
       </c>
       <c r="K30" s="12" t="n">
-        <v>649.6900000000001</v>
+        <v>486.72</v>
       </c>
       <c r="L30" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
@@ -1627,25 +1627,25 @@
         <v>17</v>
       </c>
       <c r="B31" s="12" t="n">
-        <v>68.69</v>
+        <v>68.23</v>
       </c>
       <c r="C31" s="12" t="n">
-        <v>137.38</v>
+        <v>68.23</v>
       </c>
       <c r="D31" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I31" s="11" t="n">
         <v>17</v>
       </c>
       <c r="J31" s="12" t="n">
-        <v>94.09999999999999</v>
+        <v>81.67</v>
       </c>
       <c r="K31" s="12" t="n">
-        <v>658.72</v>
+        <v>489.99</v>
       </c>
       <c r="L31" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
@@ -1653,25 +1653,25 @@
         <v>18</v>
       </c>
       <c r="B32" s="12" t="n">
-        <v>68.64</v>
+        <v>68.03</v>
       </c>
       <c r="C32" s="12" t="n">
-        <v>137.28</v>
+        <v>68.03</v>
       </c>
       <c r="D32" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I32" s="11" t="n">
         <v>18</v>
       </c>
       <c r="J32" s="12" t="n">
-        <v>95.39</v>
+        <v>82.20999999999999</v>
       </c>
       <c r="K32" s="12" t="n">
-        <v>667.75</v>
+        <v>493.26</v>
       </c>
       <c r="L32" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
@@ -1679,25 +1679,25 @@
         <v>19</v>
       </c>
       <c r="B33" s="12" t="n">
-        <v>68.59</v>
+        <v>67.83</v>
       </c>
       <c r="C33" s="12" t="n">
-        <v>137.18</v>
+        <v>67.83</v>
       </c>
       <c r="D33" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I33" s="11" t="n">
         <v>19</v>
       </c>
       <c r="J33" s="12" t="n">
-        <v>96.68000000000001</v>
+        <v>82.76000000000001</v>
       </c>
       <c r="K33" s="12" t="n">
-        <v>676.78</v>
+        <v>496.54</v>
       </c>
       <c r="L33" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34">
@@ -1705,25 +1705,25 @@
         <v>20</v>
       </c>
       <c r="B34" s="12" t="n">
-        <v>68.54000000000001</v>
+        <v>67.63</v>
       </c>
       <c r="C34" s="12" t="n">
-        <v>137.08</v>
+        <v>67.63</v>
       </c>
       <c r="D34" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I34" s="11" t="n">
         <v>20</v>
       </c>
       <c r="J34" s="12" t="n">
-        <v>97.97</v>
+        <v>83.3</v>
       </c>
       <c r="K34" s="12" t="n">
-        <v>685.8099999999999</v>
+        <v>499.81</v>
       </c>
       <c r="L34" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35">
@@ -1731,25 +1731,25 @@
         <v>21</v>
       </c>
       <c r="B35" s="12" t="n">
-        <v>68.48999999999999</v>
+        <v>67.42</v>
       </c>
       <c r="C35" s="12" t="n">
-        <v>136.98</v>
+        <v>67.42</v>
       </c>
       <c r="D35" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I35" s="11" t="n">
         <v>21</v>
       </c>
       <c r="J35" s="12" t="n">
-        <v>99.26000000000001</v>
+        <v>83.84999999999999</v>
       </c>
       <c r="K35" s="12" t="n">
-        <v>694.84</v>
+        <v>503.08</v>
       </c>
       <c r="L35" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36">
@@ -1757,25 +1757,25 @@
         <v>22</v>
       </c>
       <c r="B36" s="12" t="n">
-        <v>68.44</v>
+        <v>67.22</v>
       </c>
       <c r="C36" s="12" t="n">
-        <v>136.88</v>
+        <v>67.22</v>
       </c>
       <c r="D36" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I36" s="11" t="n">
         <v>22</v>
       </c>
       <c r="J36" s="12" t="n">
-        <v>100.55</v>
+        <v>84.39</v>
       </c>
       <c r="K36" s="12" t="n">
-        <v>703.86</v>
+        <v>506.35</v>
       </c>
       <c r="L36" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37">
@@ -1783,25 +1783,25 @@
         <v>23</v>
       </c>
       <c r="B37" s="12" t="n">
-        <v>68.39</v>
+        <v>67.02</v>
       </c>
       <c r="C37" s="12" t="n">
-        <v>136.78</v>
+        <v>67.02</v>
       </c>
       <c r="D37" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I37" s="11" t="n">
         <v>23</v>
       </c>
       <c r="J37" s="12" t="n">
-        <v>101.84</v>
+        <v>84.94</v>
       </c>
       <c r="K37" s="12" t="n">
-        <v>712.89</v>
+        <v>509.62</v>
       </c>
       <c r="L37" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38">
@@ -1809,25 +1809,25 @@
         <v>24</v>
       </c>
       <c r="B38" s="12" t="n">
-        <v>68.34</v>
+        <v>66.81999999999999</v>
       </c>
       <c r="C38" s="12" t="n">
-        <v>136.68</v>
+        <v>66.81999999999999</v>
       </c>
       <c r="D38" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I38" s="11" t="n">
         <v>24</v>
       </c>
       <c r="J38" s="12" t="n">
-        <v>103.13</v>
+        <v>85.48</v>
       </c>
       <c r="K38" s="12" t="n">
-        <v>721.92</v>
+        <v>512.89</v>
       </c>
       <c r="L38" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39">
@@ -1835,25 +1835,25 @@
         <v>25</v>
       </c>
       <c r="B39" s="12" t="n">
-        <v>68.29000000000001</v>
+        <v>66.61</v>
       </c>
       <c r="C39" s="12" t="n">
-        <v>136.58</v>
+        <v>66.61</v>
       </c>
       <c r="D39" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I39" s="11" t="n">
         <v>25</v>
       </c>
       <c r="J39" s="12" t="n">
-        <v>104.42</v>
+        <v>86.03</v>
       </c>
       <c r="K39" s="12" t="n">
-        <v>730.95</v>
+        <v>516.16</v>
       </c>
       <c r="L39" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40">
@@ -1861,25 +1861,25 @@
         <v>26</v>
       </c>
       <c r="B40" s="12" t="n">
-        <v>68.23999999999999</v>
+        <v>66.41</v>
       </c>
       <c r="C40" s="12" t="n">
-        <v>136.48</v>
+        <v>66.41</v>
       </c>
       <c r="D40" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I40" s="11" t="n">
         <v>26</v>
       </c>
       <c r="J40" s="12" t="n">
-        <v>105.71</v>
+        <v>86.56999999999999</v>
       </c>
       <c r="K40" s="12" t="n">
-        <v>739.98</v>
+        <v>519.4299999999999</v>
       </c>
       <c r="L40" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41">
@@ -1887,25 +1887,25 @@
         <v>27</v>
       </c>
       <c r="B41" s="12" t="n">
-        <v>68.19</v>
+        <v>66.20999999999999</v>
       </c>
       <c r="C41" s="12" t="n">
-        <v>136.38</v>
+        <v>66.20999999999999</v>
       </c>
       <c r="D41" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I41" s="11" t="n">
         <v>27</v>
       </c>
       <c r="J41" s="12" t="n">
-        <v>107</v>
+        <v>87.12</v>
       </c>
       <c r="K41" s="12" t="n">
-        <v>749.01</v>
+        <v>522.71</v>
       </c>
       <c r="L41" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42">
@@ -1913,25 +1913,25 @@
         <v>28</v>
       </c>
       <c r="B42" s="12" t="n">
-        <v>68.14</v>
+        <v>66.01000000000001</v>
       </c>
       <c r="C42" s="12" t="n">
-        <v>136.28</v>
+        <v>66.01000000000001</v>
       </c>
       <c r="D42" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I42" s="11" t="n">
         <v>28</v>
       </c>
       <c r="J42" s="12" t="n">
-        <v>108.29</v>
+        <v>87.66</v>
       </c>
       <c r="K42" s="12" t="n">
-        <v>758.04</v>
+        <v>525.98</v>
       </c>
       <c r="L42" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43">
@@ -1939,25 +1939,25 @@
         <v>29</v>
       </c>
       <c r="B43" s="12" t="n">
-        <v>68.09</v>
+        <v>65.8</v>
       </c>
       <c r="C43" s="12" t="n">
-        <v>136.18</v>
+        <v>65.8</v>
       </c>
       <c r="D43" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I43" s="11" t="n">
         <v>29</v>
       </c>
       <c r="J43" s="12" t="n">
-        <v>109.58</v>
+        <v>88.20999999999999</v>
       </c>
       <c r="K43" s="12" t="n">
-        <v>767.0700000000001</v>
+        <v>529.25</v>
       </c>
       <c r="L43" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
@@ -1965,25 +1965,25 @@
         <v>30</v>
       </c>
       <c r="B44" s="12" t="n">
-        <v>68.04000000000001</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="C44" s="12" t="n">
-        <v>136.08</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="D44" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I44" s="11" t="n">
         <v>30</v>
       </c>
       <c r="J44" s="12" t="n">
-        <v>110.87</v>
+        <v>88.75</v>
       </c>
       <c r="K44" s="12" t="n">
-        <v>776.1</v>
+        <v>532.52</v>
       </c>
       <c r="L44" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove 2% profit restriction on sell and widen buy grid down to lower target price
</commit_message>
<xml_diff>
--- a/vr_portfolio_log.xlsx
+++ b/vr_portfolio_log.xlsx
@@ -738,7 +738,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -798,10 +798,10 @@
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="B4" s="3" t="n">
-        <v>19878.43</v>
+        <v>9364.99</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>14882.92</v>
+        <v>4369.48</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>4995.51</v>
@@ -810,14 +810,14 @@
         <v>4369.48</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>4157.246639999999</v>
+        <v>4138.67635</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>5624.510159999999</v>
+        <v>5599.385649999999</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>HOLD</t>
         </is>
       </c>
     </row>
@@ -1031,19 +1031,19 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>70.76000000000001</v>
+        <v>70.87</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>213</v>
+        <v>200</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>14882.92</v>
+        <v>4369.48</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>4995.51</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>19878.43</v>
+        <v>9364.99</v>
       </c>
       <c r="H10" s="6" t="n">
         <v>4369.48</v>
@@ -1057,24 +1057,24 @@
         </is>
       </c>
       <c r="K10" s="8" t="n">
-        <v>0.1193</v>
+        <v>0.1143</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>4890.88</v>
+        <v>4869.03</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>4157.25</v>
+        <v>4138.68</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>5624.51</v>
-      </c>
-      <c r="O10" s="18" t="inlineStr">
-        <is>
-          <t>SELL</t>
+        <v>5599.39</v>
+      </c>
+      <c r="O10" s="14" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="P10" s="6" t="n">
-        <v>9992.040000000001</v>
+        <v>499.55</v>
       </c>
     </row>
     <row r="11">
@@ -1220,10 +1220,10 @@
         <v>1</v>
       </c>
       <c r="B15" s="12" t="n">
-        <v>68.08</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>68.08</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="D15" s="13" t="n">
         <v>1</v>
@@ -1232,13 +1232,13 @@
         <v>1</v>
       </c>
       <c r="J15" s="12" t="n">
-        <v>72.66</v>
+        <v>75.48</v>
       </c>
       <c r="K15" s="12" t="n">
-        <v>508.59</v>
+        <v>452.9</v>
       </c>
       <c r="L15" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
@@ -1246,10 +1246,10 @@
         <v>2</v>
       </c>
       <c r="B16" s="12" t="n">
-        <v>66.41</v>
+        <v>69.53</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>66.41</v>
+        <v>69.53</v>
       </c>
       <c r="D16" s="13" t="n">
         <v>1</v>
@@ -1258,13 +1258,13 @@
         <v>2</v>
       </c>
       <c r="J16" s="12" t="n">
-        <v>73.14</v>
+        <v>78.7</v>
       </c>
       <c r="K16" s="12" t="n">
-        <v>511.96</v>
+        <v>472.22</v>
       </c>
       <c r="L16" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
@@ -1272,10 +1272,10 @@
         <v>3</v>
       </c>
       <c r="B17" s="12" t="n">
-        <v>64.73</v>
+        <v>68.45</v>
       </c>
       <c r="C17" s="12" t="n">
-        <v>64.73</v>
+        <v>68.45</v>
       </c>
       <c r="D17" s="13" t="n">
         <v>1</v>
@@ -1284,13 +1284,13 @@
         <v>3</v>
       </c>
       <c r="J17" s="12" t="n">
-        <v>73.62</v>
+        <v>82.06</v>
       </c>
       <c r="K17" s="12" t="n">
-        <v>515.33</v>
+        <v>492.35</v>
       </c>
       <c r="L17" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -1298,10 +1298,10 @@
         <v>4</v>
       </c>
       <c r="B18" s="12" t="n">
-        <v>63.06</v>
+        <v>67.38</v>
       </c>
       <c r="C18" s="12" t="n">
-        <v>63.06</v>
+        <v>67.38</v>
       </c>
       <c r="D18" s="13" t="n">
         <v>1</v>
@@ -1310,13 +1310,13 @@
         <v>4</v>
       </c>
       <c r="J18" s="12" t="n">
-        <v>74.09999999999999</v>
+        <v>85.56</v>
       </c>
       <c r="K18" s="12" t="n">
-        <v>518.7</v>
+        <v>513.35</v>
       </c>
       <c r="L18" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
@@ -1324,25 +1324,25 @@
         <v>5</v>
       </c>
       <c r="B19" s="12" t="n">
-        <v>61.38</v>
+        <v>66.3</v>
       </c>
       <c r="C19" s="12" t="n">
-        <v>122.76</v>
+        <v>66.3</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I19" s="11" t="n">
         <v>5</v>
       </c>
       <c r="J19" s="12" t="n">
-        <v>74.58</v>
+        <v>89.20999999999999</v>
       </c>
       <c r="K19" s="12" t="n">
-        <v>522.0700000000001</v>
+        <v>535.24</v>
       </c>
       <c r="L19" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -1350,25 +1350,25 @@
         <v>6</v>
       </c>
       <c r="B20" s="12" t="n">
-        <v>59.71</v>
+        <v>65.23</v>
       </c>
       <c r="C20" s="12" t="n">
-        <v>119.41</v>
+        <v>65.23</v>
       </c>
       <c r="D20" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I20" s="11" t="n">
         <v>6</v>
       </c>
       <c r="J20" s="12" t="n">
-        <v>75.06</v>
+        <v>93.01000000000001</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>525.4400000000001</v>
+        <v>558.0599999999999</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -1376,25 +1376,25 @@
         <v>7</v>
       </c>
       <c r="B21" s="12" t="n">
-        <v>58.03</v>
+        <v>64.15000000000001</v>
       </c>
       <c r="C21" s="12" t="n">
-        <v>116.06</v>
+        <v>64.15000000000001</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I21" s="11" t="n">
         <v>7</v>
       </c>
       <c r="J21" s="12" t="n">
-        <v>75.54000000000001</v>
+        <v>96.98</v>
       </c>
       <c r="K21" s="12" t="n">
-        <v>528.8</v>
+        <v>581.86</v>
       </c>
       <c r="L21" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
@@ -1402,25 +1402,25 @@
         <v>8</v>
       </c>
       <c r="B22" s="12" t="n">
-        <v>56.35</v>
+        <v>63.08</v>
       </c>
       <c r="C22" s="12" t="n">
-        <v>112.71</v>
+        <v>63.08</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I22" s="11" t="n">
         <v>8</v>
       </c>
       <c r="J22" s="12" t="n">
-        <v>76.02</v>
+        <v>101.11</v>
       </c>
       <c r="K22" s="12" t="n">
-        <v>532.17</v>
+        <v>606.67</v>
       </c>
       <c r="L22" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23">
@@ -1428,10 +1428,10 @@
         <v>9</v>
       </c>
       <c r="B23" s="12" t="n">
-        <v>54.68</v>
+        <v>62</v>
       </c>
       <c r="C23" s="12" t="n">
-        <v>109.36</v>
+        <v>124.01</v>
       </c>
       <c r="D23" s="13" t="n">
         <v>2</v>
@@ -1440,13 +1440,13 @@
         <v>9</v>
       </c>
       <c r="J23" s="12" t="n">
-        <v>76.51000000000001</v>
+        <v>105.42</v>
       </c>
       <c r="K23" s="12" t="n">
-        <v>535.54</v>
+        <v>632.54</v>
       </c>
       <c r="L23" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
@@ -1454,10 +1454,10 @@
         <v>10</v>
       </c>
       <c r="B24" s="12" t="n">
-        <v>53</v>
+        <v>60.93</v>
       </c>
       <c r="C24" s="12" t="n">
-        <v>106</v>
+        <v>121.86</v>
       </c>
       <c r="D24" s="13" t="n">
         <v>2</v>
@@ -1466,13 +1466,13 @@
         <v>10</v>
       </c>
       <c r="J24" s="12" t="n">
-        <v>76.98999999999999</v>
+        <v>109.92</v>
       </c>
       <c r="K24" s="12" t="n">
-        <v>538.91</v>
+        <v>659.52</v>
       </c>
       <c r="L24" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -1480,10 +1480,10 @@
         <v>11</v>
       </c>
       <c r="B25" s="12" t="n">
-        <v>51.33</v>
+        <v>59.85</v>
       </c>
       <c r="C25" s="12" t="n">
-        <v>102.65</v>
+        <v>119.71</v>
       </c>
       <c r="D25" s="13" t="n">
         <v>2</v>
@@ -1492,13 +1492,13 @@
         <v>11</v>
       </c>
       <c r="J25" s="12" t="n">
-        <v>77.47</v>
+        <v>114.61</v>
       </c>
       <c r="K25" s="12" t="n">
-        <v>542.28</v>
+        <v>687.64</v>
       </c>
       <c r="L25" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -1506,10 +1506,10 @@
         <v>12</v>
       </c>
       <c r="B26" s="12" t="n">
-        <v>49.65</v>
+        <v>58.78</v>
       </c>
       <c r="C26" s="12" t="n">
-        <v>99.3</v>
+        <v>117.56</v>
       </c>
       <c r="D26" s="13" t="n">
         <v>2</v>
@@ -1518,13 +1518,13 @@
         <v>12</v>
       </c>
       <c r="J26" s="12" t="n">
-        <v>77.95</v>
+        <v>119.49</v>
       </c>
       <c r="K26" s="12" t="n">
-        <v>545.64</v>
+        <v>716.96</v>
       </c>
       <c r="L26" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
@@ -1532,10 +1532,10 @@
         <v>13</v>
       </c>
       <c r="B27" s="12" t="n">
-        <v>47.97</v>
+        <v>57.7</v>
       </c>
       <c r="C27" s="12" t="n">
-        <v>95.95</v>
+        <v>115.4</v>
       </c>
       <c r="D27" s="13" t="n">
         <v>2</v>
@@ -1544,13 +1544,13 @@
         <v>13</v>
       </c>
       <c r="J27" s="12" t="n">
-        <v>78.43000000000001</v>
+        <v>124.59</v>
       </c>
       <c r="K27" s="12" t="n">
-        <v>549.01</v>
+        <v>747.54</v>
       </c>
       <c r="L27" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28">
@@ -1558,10 +1558,10 @@
         <v>14</v>
       </c>
       <c r="B28" s="12" t="n">
-        <v>46.3</v>
+        <v>56.63</v>
       </c>
       <c r="C28" s="12" t="n">
-        <v>92.59999999999999</v>
+        <v>113.25</v>
       </c>
       <c r="D28" s="13" t="n">
         <v>2</v>
@@ -1570,13 +1570,13 @@
         <v>14</v>
       </c>
       <c r="J28" s="12" t="n">
-        <v>78.91</v>
+        <v>129.9</v>
       </c>
       <c r="K28" s="12" t="n">
-        <v>552.38</v>
+        <v>779.42</v>
       </c>
       <c r="L28" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
@@ -1584,10 +1584,10 @@
         <v>15</v>
       </c>
       <c r="B29" s="12" t="n">
-        <v>44.62</v>
+        <v>55.55</v>
       </c>
       <c r="C29" s="12" t="n">
-        <v>89.25</v>
+        <v>111.1</v>
       </c>
       <c r="D29" s="13" t="n">
         <v>2</v>
@@ -1596,13 +1596,13 @@
         <v>15</v>
       </c>
       <c r="J29" s="12" t="n">
-        <v>79.39</v>
+        <v>135.44</v>
       </c>
       <c r="K29" s="12" t="n">
-        <v>555.75</v>
+        <v>812.65</v>
       </c>
       <c r="L29" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
@@ -1610,10 +1610,10 @@
         <v>16</v>
       </c>
       <c r="B30" s="12" t="n">
-        <v>42.95</v>
+        <v>54.48</v>
       </c>
       <c r="C30" s="12" t="n">
-        <v>85.89</v>
+        <v>108.95</v>
       </c>
       <c r="D30" s="13" t="n">
         <v>2</v>
@@ -1622,13 +1622,13 @@
         <v>16</v>
       </c>
       <c r="J30" s="12" t="n">
-        <v>79.87</v>
+        <v>141.22</v>
       </c>
       <c r="K30" s="12" t="n">
-        <v>559.12</v>
+        <v>847.3099999999999</v>
       </c>
       <c r="L30" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
@@ -1636,25 +1636,25 @@
         <v>17</v>
       </c>
       <c r="B31" s="12" t="n">
-        <v>41.27</v>
+        <v>53.4</v>
       </c>
       <c r="C31" s="12" t="n">
-        <v>123.81</v>
+        <v>106.8</v>
       </c>
       <c r="D31" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I31" s="11" t="n">
         <v>17</v>
       </c>
       <c r="J31" s="12" t="n">
-        <v>80.36</v>
+        <v>147.24</v>
       </c>
       <c r="K31" s="12" t="n">
-        <v>562.49</v>
+        <v>883.4400000000001</v>
       </c>
       <c r="L31" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
@@ -1662,25 +1662,25 @@
         <v>18</v>
       </c>
       <c r="B32" s="12" t="n">
-        <v>39.6</v>
+        <v>52.33</v>
       </c>
       <c r="C32" s="12" t="n">
-        <v>118.79</v>
+        <v>104.65</v>
       </c>
       <c r="D32" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I32" s="11" t="n">
         <v>18</v>
       </c>
       <c r="J32" s="12" t="n">
-        <v>80.84</v>
+        <v>153.52</v>
       </c>
       <c r="K32" s="12" t="n">
-        <v>565.85</v>
+        <v>921.11</v>
       </c>
       <c r="L32" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
@@ -1688,25 +1688,25 @@
         <v>19</v>
       </c>
       <c r="B33" s="12" t="n">
-        <v>37.92</v>
+        <v>51.25</v>
       </c>
       <c r="C33" s="12" t="n">
-        <v>113.76</v>
+        <v>102.5</v>
       </c>
       <c r="D33" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I33" s="11" t="n">
         <v>19</v>
       </c>
       <c r="J33" s="12" t="n">
-        <v>81.31999999999999</v>
+        <v>160.06</v>
       </c>
       <c r="K33" s="12" t="n">
-        <v>569.22</v>
+        <v>960.39</v>
       </c>
       <c r="L33" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34">
@@ -1714,25 +1714,25 @@
         <v>20</v>
       </c>
       <c r="B34" s="12" t="n">
-        <v>36.24</v>
+        <v>50.18</v>
       </c>
       <c r="C34" s="12" t="n">
-        <v>108.73</v>
+        <v>100.35</v>
       </c>
       <c r="D34" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I34" s="11" t="n">
         <v>20</v>
       </c>
       <c r="J34" s="12" t="n">
-        <v>81.8</v>
+        <v>166.89</v>
       </c>
       <c r="K34" s="12" t="n">
-        <v>572.59</v>
+        <v>1001.34</v>
       </c>
       <c r="L34" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35">
@@ -1740,25 +1740,25 @@
         <v>21</v>
       </c>
       <c r="B35" s="12" t="n">
-        <v>34.57</v>
+        <v>49.1</v>
       </c>
       <c r="C35" s="12" t="n">
-        <v>103.7</v>
+        <v>98.2</v>
       </c>
       <c r="D35" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I35" s="11" t="n">
         <v>21</v>
       </c>
       <c r="J35" s="12" t="n">
-        <v>82.28</v>
+        <v>174.01</v>
       </c>
       <c r="K35" s="12" t="n">
-        <v>575.96</v>
+        <v>1044.04</v>
       </c>
       <c r="L35" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36">
@@ -1766,25 +1766,25 @@
         <v>22</v>
       </c>
       <c r="B36" s="12" t="n">
-        <v>32.89</v>
+        <v>48.03</v>
       </c>
       <c r="C36" s="12" t="n">
-        <v>98.68000000000001</v>
+        <v>96.05</v>
       </c>
       <c r="D36" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I36" s="11" t="n">
         <v>22</v>
       </c>
       <c r="J36" s="12" t="n">
-        <v>82.76000000000001</v>
+        <v>181.43</v>
       </c>
       <c r="K36" s="12" t="n">
-        <v>579.33</v>
+        <v>1088.56</v>
       </c>
       <c r="L36" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37">
@@ -1792,25 +1792,25 @@
         <v>23</v>
       </c>
       <c r="B37" s="12" t="n">
-        <v>31.22</v>
+        <v>46.95</v>
       </c>
       <c r="C37" s="12" t="n">
-        <v>124.87</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="D37" s="13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I37" s="11" t="n">
         <v>23</v>
       </c>
       <c r="J37" s="12" t="n">
-        <v>83.23999999999999</v>
+        <v>189.16</v>
       </c>
       <c r="K37" s="12" t="n">
-        <v>582.6900000000001</v>
+        <v>1134.98</v>
       </c>
       <c r="L37" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38">
@@ -1818,25 +1818,25 @@
         <v>24</v>
       </c>
       <c r="B38" s="12" t="n">
-        <v>29.54</v>
+        <v>45.88</v>
       </c>
       <c r="C38" s="12" t="n">
-        <v>118.16</v>
+        <v>91.75</v>
       </c>
       <c r="D38" s="13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I38" s="11" t="n">
         <v>24</v>
       </c>
       <c r="J38" s="12" t="n">
-        <v>83.72</v>
+        <v>197.23</v>
       </c>
       <c r="K38" s="12" t="n">
-        <v>586.0599999999999</v>
+        <v>1183.38</v>
       </c>
       <c r="L38" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39">
@@ -1844,25 +1844,25 @@
         <v>25</v>
       </c>
       <c r="B39" s="12" t="n">
-        <v>27.87</v>
+        <v>44.8</v>
       </c>
       <c r="C39" s="12" t="n">
-        <v>111.46</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="D39" s="13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I39" s="11" t="n">
         <v>25</v>
       </c>
       <c r="J39" s="12" t="n">
-        <v>84.2</v>
+        <v>205.64</v>
       </c>
       <c r="K39" s="12" t="n">
-        <v>589.4299999999999</v>
+        <v>1233.85</v>
       </c>
       <c r="L39" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40">
@@ -1870,25 +1870,25 @@
         <v>26</v>
       </c>
       <c r="B40" s="12" t="n">
-        <v>26.19</v>
+        <v>43.72</v>
       </c>
       <c r="C40" s="12" t="n">
-        <v>104.76</v>
+        <v>87.45</v>
       </c>
       <c r="D40" s="13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I40" s="11" t="n">
         <v>26</v>
       </c>
       <c r="J40" s="12" t="n">
-        <v>84.69</v>
+        <v>214.41</v>
       </c>
       <c r="K40" s="12" t="n">
-        <v>592.8</v>
+        <v>1286.46</v>
       </c>
       <c r="L40" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41">
@@ -1896,25 +1896,25 @@
         <v>27</v>
       </c>
       <c r="B41" s="12" t="n">
-        <v>24.51</v>
+        <v>42.65</v>
       </c>
       <c r="C41" s="12" t="n">
-        <v>122.57</v>
+        <v>85.3</v>
       </c>
       <c r="D41" s="13" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I41" s="11" t="n">
         <v>27</v>
       </c>
       <c r="J41" s="12" t="n">
-        <v>85.17</v>
+        <v>223.55</v>
       </c>
       <c r="K41" s="12" t="n">
-        <v>596.17</v>
+        <v>1341.32</v>
       </c>
       <c r="L41" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42">
@@ -1922,25 +1922,25 @@
         <v>28</v>
       </c>
       <c r="B42" s="12" t="n">
-        <v>22.84</v>
+        <v>41.57</v>
       </c>
       <c r="C42" s="12" t="n">
-        <v>114.19</v>
+        <v>124.72</v>
       </c>
       <c r="D42" s="13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I42" s="11" t="n">
         <v>28</v>
       </c>
       <c r="J42" s="12" t="n">
-        <v>85.65000000000001</v>
+        <v>233.09</v>
       </c>
       <c r="K42" s="12" t="n">
-        <v>599.54</v>
+        <v>1398.52</v>
       </c>
       <c r="L42" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43">
@@ -1948,25 +1948,25 @@
         <v>29</v>
       </c>
       <c r="B43" s="12" t="n">
-        <v>21.16</v>
+        <v>40.5</v>
       </c>
       <c r="C43" s="12" t="n">
-        <v>105.81</v>
+        <v>121.5</v>
       </c>
       <c r="D43" s="13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I43" s="11" t="n">
         <v>29</v>
       </c>
       <c r="J43" s="12" t="n">
-        <v>86.13</v>
+        <v>243.03</v>
       </c>
       <c r="K43" s="12" t="n">
-        <v>602.9</v>
+        <v>1458.15</v>
       </c>
       <c r="L43" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
@@ -1974,25 +1974,25 @@
         <v>30</v>
       </c>
       <c r="B44" s="12" t="n">
-        <v>19.49</v>
+        <v>39.42</v>
       </c>
       <c r="C44" s="12" t="n">
-        <v>116.92</v>
+        <v>118.27</v>
       </c>
       <c r="D44" s="13" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I44" s="11" t="n">
         <v>30</v>
       </c>
       <c r="J44" s="12" t="n">
-        <v>86.61</v>
+        <v>253.39</v>
       </c>
       <c r="K44" s="12" t="n">
-        <v>606.27</v>
+        <v>1520.33</v>
       </c>
       <c r="L44" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix fallback to use user actual TQQQ qty (51) and avg price (4.08) from state
</commit_message>
<xml_diff>
--- a/vr_portfolio_log.xlsx
+++ b/vr_portfolio_log.xlsx
@@ -735,10 +735,10 @@
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -798,26 +798,26 @@
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="B4" s="3" t="n">
-        <v>9364.99</v>
+        <v>6661.699922180176</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>4369.48</v>
+        <v>3549.599922180176</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>4995.51</v>
+        <v>3112.1</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>4369.48</v>
+        <v>4058.27</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>4138.67635</v>
+        <v>3714.058</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>5599.385649999999</v>
+        <v>5024.901999999999</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>BUY</t>
         </is>
       </c>
     </row>
@@ -1031,50 +1031,50 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>70.87</v>
+        <v>74.08</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>200</v>
+        <v>51</v>
       </c>
       <c r="E10" s="6" t="n">
+        <v>3549.6</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>3112.1</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>6661.7</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>4058.27</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>0.7669</v>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>/10</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="n">
+        <v>0.0767</v>
+      </c>
+      <c r="L10" s="6" t="n">
         <v>4369.48</v>
       </c>
-      <c r="F10" s="6" t="n">
-        <v>4995.51</v>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>9364.99</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>4369.48</v>
-      </c>
-      <c r="I10" s="8" t="n">
-        <v>1.1433</v>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>/10</t>
-        </is>
-      </c>
-      <c r="K10" s="8" t="n">
-        <v>0.1143</v>
-      </c>
-      <c r="L10" s="6" t="n">
-        <v>4869.03</v>
-      </c>
       <c r="M10" s="6" t="n">
-        <v>4138.68</v>
+        <v>3714.06</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>5599.39</v>
-      </c>
-      <c r="O10" s="14" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>5024.9</v>
+      </c>
+      <c r="O10" s="9" t="inlineStr">
+        <is>
+          <t>BUY</t>
         </is>
       </c>
       <c r="P10" s="6" t="n">
-        <v>499.55</v>
+        <v>819.88</v>
       </c>
     </row>
     <row r="11">
@@ -1220,10 +1220,10 @@
         <v>1</v>
       </c>
       <c r="B15" s="12" t="n">
-        <v>70.59999999999999</v>
+        <v>68.56</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>70.59999999999999</v>
+        <v>68.56</v>
       </c>
       <c r="D15" s="13" t="n">
         <v>1</v>
@@ -1232,13 +1232,13 @@
         <v>1</v>
       </c>
       <c r="J15" s="12" t="n">
-        <v>75.48</v>
+        <v>73.29000000000001</v>
       </c>
       <c r="K15" s="12" t="n">
-        <v>452.9</v>
+        <v>73.29000000000001</v>
       </c>
       <c r="L15" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1246,10 +1246,10 @@
         <v>2</v>
       </c>
       <c r="B16" s="12" t="n">
-        <v>69.53</v>
+        <v>67.51000000000001</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>69.53</v>
+        <v>67.51000000000001</v>
       </c>
       <c r="D16" s="13" t="n">
         <v>1</v>
@@ -1258,13 +1258,13 @@
         <v>2</v>
       </c>
       <c r="J16" s="12" t="n">
-        <v>78.7</v>
+        <v>76.42</v>
       </c>
       <c r="K16" s="12" t="n">
-        <v>472.22</v>
+        <v>76.42</v>
       </c>
       <c r="L16" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -1272,10 +1272,10 @@
         <v>3</v>
       </c>
       <c r="B17" s="12" t="n">
-        <v>68.45</v>
+        <v>66.47</v>
       </c>
       <c r="C17" s="12" t="n">
-        <v>68.45</v>
+        <v>66.47</v>
       </c>
       <c r="D17" s="13" t="n">
         <v>1</v>
@@ -1284,13 +1284,13 @@
         <v>3</v>
       </c>
       <c r="J17" s="12" t="n">
-        <v>82.06</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="K17" s="12" t="n">
-        <v>492.35</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="L17" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1298,10 +1298,10 @@
         <v>4</v>
       </c>
       <c r="B18" s="12" t="n">
-        <v>67.38</v>
+        <v>65.42</v>
       </c>
       <c r="C18" s="12" t="n">
-        <v>67.38</v>
+        <v>65.42</v>
       </c>
       <c r="D18" s="13" t="n">
         <v>1</v>
@@ -1310,13 +1310,13 @@
         <v>4</v>
       </c>
       <c r="J18" s="12" t="n">
-        <v>85.56</v>
+        <v>83.08</v>
       </c>
       <c r="K18" s="12" t="n">
-        <v>513.35</v>
+        <v>83.08</v>
       </c>
       <c r="L18" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -1324,10 +1324,10 @@
         <v>5</v>
       </c>
       <c r="B19" s="12" t="n">
-        <v>66.3</v>
+        <v>64.38</v>
       </c>
       <c r="C19" s="12" t="n">
-        <v>66.3</v>
+        <v>64.38</v>
       </c>
       <c r="D19" s="13" t="n">
         <v>1</v>
@@ -1336,13 +1336,13 @@
         <v>5</v>
       </c>
       <c r="J19" s="12" t="n">
-        <v>89.20999999999999</v>
+        <v>86.62</v>
       </c>
       <c r="K19" s="12" t="n">
-        <v>535.24</v>
+        <v>86.62</v>
       </c>
       <c r="L19" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1350,10 +1350,10 @@
         <v>6</v>
       </c>
       <c r="B20" s="12" t="n">
-        <v>65.23</v>
+        <v>63.34</v>
       </c>
       <c r="C20" s="12" t="n">
-        <v>65.23</v>
+        <v>63.34</v>
       </c>
       <c r="D20" s="13" t="n">
         <v>1</v>
@@ -1362,13 +1362,13 @@
         <v>6</v>
       </c>
       <c r="J20" s="12" t="n">
-        <v>93.01000000000001</v>
+        <v>90.31</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>558.0599999999999</v>
+        <v>90.31</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1376,10 +1376,10 @@
         <v>7</v>
       </c>
       <c r="B21" s="12" t="n">
-        <v>64.15000000000001</v>
+        <v>62.29</v>
       </c>
       <c r="C21" s="12" t="n">
-        <v>64.15000000000001</v>
+        <v>62.29</v>
       </c>
       <c r="D21" s="13" t="n">
         <v>1</v>
@@ -1388,13 +1388,13 @@
         <v>7</v>
       </c>
       <c r="J21" s="12" t="n">
-        <v>96.98</v>
+        <v>94.16</v>
       </c>
       <c r="K21" s="12" t="n">
-        <v>581.86</v>
+        <v>94.16</v>
       </c>
       <c r="L21" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1402,10 +1402,10 @@
         <v>8</v>
       </c>
       <c r="B22" s="12" t="n">
-        <v>63.08</v>
+        <v>61.25</v>
       </c>
       <c r="C22" s="12" t="n">
-        <v>63.08</v>
+        <v>61.25</v>
       </c>
       <c r="D22" s="13" t="n">
         <v>1</v>
@@ -1414,13 +1414,13 @@
         <v>8</v>
       </c>
       <c r="J22" s="12" t="n">
-        <v>101.11</v>
+        <v>98.18000000000001</v>
       </c>
       <c r="K22" s="12" t="n">
-        <v>606.67</v>
+        <v>98.18000000000001</v>
       </c>
       <c r="L22" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -1428,25 +1428,25 @@
         <v>9</v>
       </c>
       <c r="B23" s="12" t="n">
-        <v>62</v>
+        <v>60.2</v>
       </c>
       <c r="C23" s="12" t="n">
-        <v>124.01</v>
+        <v>60.2</v>
       </c>
       <c r="D23" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I23" s="11" t="n">
         <v>9</v>
       </c>
       <c r="J23" s="12" t="n">
-        <v>105.42</v>
+        <v>102.36</v>
       </c>
       <c r="K23" s="12" t="n">
-        <v>632.54</v>
+        <v>102.36</v>
       </c>
       <c r="L23" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1454,25 +1454,25 @@
         <v>10</v>
       </c>
       <c r="B24" s="12" t="n">
-        <v>60.93</v>
+        <v>59.16</v>
       </c>
       <c r="C24" s="12" t="n">
-        <v>121.86</v>
+        <v>59.16</v>
       </c>
       <c r="D24" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I24" s="11" t="n">
         <v>10</v>
       </c>
       <c r="J24" s="12" t="n">
-        <v>109.92</v>
+        <v>106.73</v>
       </c>
       <c r="K24" s="12" t="n">
-        <v>659.52</v>
+        <v>106.73</v>
       </c>
       <c r="L24" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1480,25 +1480,25 @@
         <v>11</v>
       </c>
       <c r="B25" s="12" t="n">
-        <v>59.85</v>
+        <v>58.12</v>
       </c>
       <c r="C25" s="12" t="n">
-        <v>119.71</v>
+        <v>58.12</v>
       </c>
       <c r="D25" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I25" s="11" t="n">
         <v>11</v>
       </c>
       <c r="J25" s="12" t="n">
-        <v>114.61</v>
+        <v>111.28</v>
       </c>
       <c r="K25" s="12" t="n">
-        <v>687.64</v>
+        <v>111.28</v>
       </c>
       <c r="L25" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -1506,25 +1506,25 @@
         <v>12</v>
       </c>
       <c r="B26" s="12" t="n">
-        <v>58.78</v>
+        <v>57.07</v>
       </c>
       <c r="C26" s="12" t="n">
-        <v>117.56</v>
+        <v>57.07</v>
       </c>
       <c r="D26" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I26" s="11" t="n">
         <v>12</v>
       </c>
       <c r="J26" s="12" t="n">
-        <v>119.49</v>
+        <v>116.03</v>
       </c>
       <c r="K26" s="12" t="n">
-        <v>716.96</v>
+        <v>116.03</v>
       </c>
       <c r="L26" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -1532,25 +1532,25 @@
         <v>13</v>
       </c>
       <c r="B27" s="12" t="n">
-        <v>57.7</v>
+        <v>56.03</v>
       </c>
       <c r="C27" s="12" t="n">
-        <v>115.4</v>
+        <v>56.03</v>
       </c>
       <c r="D27" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I27" s="11" t="n">
         <v>13</v>
       </c>
       <c r="J27" s="12" t="n">
-        <v>124.59</v>
+        <v>120.97</v>
       </c>
       <c r="K27" s="12" t="n">
-        <v>747.54</v>
+        <v>120.97</v>
       </c>
       <c r="L27" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -1558,25 +1558,25 @@
         <v>14</v>
       </c>
       <c r="B28" s="12" t="n">
-        <v>56.63</v>
+        <v>54.98</v>
       </c>
       <c r="C28" s="12" t="n">
-        <v>113.25</v>
+        <v>54.98</v>
       </c>
       <c r="D28" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I28" s="11" t="n">
         <v>14</v>
       </c>
       <c r="J28" s="12" t="n">
-        <v>129.9</v>
+        <v>126.13</v>
       </c>
       <c r="K28" s="12" t="n">
-        <v>779.42</v>
+        <v>126.13</v>
       </c>
       <c r="L28" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -1584,25 +1584,25 @@
         <v>15</v>
       </c>
       <c r="B29" s="12" t="n">
-        <v>55.55</v>
+        <v>53.94</v>
       </c>
       <c r="C29" s="12" t="n">
-        <v>111.1</v>
+        <v>53.94</v>
       </c>
       <c r="D29" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I29" s="11" t="n">
         <v>15</v>
       </c>
       <c r="J29" s="12" t="n">
-        <v>135.44</v>
+        <v>131.51</v>
       </c>
       <c r="K29" s="12" t="n">
-        <v>812.65</v>
+        <v>131.51</v>
       </c>
       <c r="L29" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -1610,25 +1610,25 @@
         <v>16</v>
       </c>
       <c r="B30" s="12" t="n">
-        <v>54.48</v>
+        <v>52.9</v>
       </c>
       <c r="C30" s="12" t="n">
-        <v>108.95</v>
+        <v>52.9</v>
       </c>
       <c r="D30" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I30" s="11" t="n">
         <v>16</v>
       </c>
       <c r="J30" s="12" t="n">
-        <v>141.22</v>
+        <v>137.12</v>
       </c>
       <c r="K30" s="12" t="n">
-        <v>847.3099999999999</v>
+        <v>137.12</v>
       </c>
       <c r="L30" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -1636,25 +1636,25 @@
         <v>17</v>
       </c>
       <c r="B31" s="12" t="n">
-        <v>53.4</v>
+        <v>51.85</v>
       </c>
       <c r="C31" s="12" t="n">
-        <v>106.8</v>
+        <v>51.85</v>
       </c>
       <c r="D31" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I31" s="11" t="n">
         <v>17</v>
       </c>
       <c r="J31" s="12" t="n">
-        <v>147.24</v>
+        <v>142.97</v>
       </c>
       <c r="K31" s="12" t="n">
-        <v>883.4400000000001</v>
+        <v>142.97</v>
       </c>
       <c r="L31" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -1662,25 +1662,25 @@
         <v>18</v>
       </c>
       <c r="B32" s="12" t="n">
-        <v>52.33</v>
+        <v>50.81</v>
       </c>
       <c r="C32" s="12" t="n">
-        <v>104.65</v>
+        <v>50.81</v>
       </c>
       <c r="D32" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I32" s="11" t="n">
         <v>18</v>
       </c>
       <c r="J32" s="12" t="n">
-        <v>153.52</v>
+        <v>149.06</v>
       </c>
       <c r="K32" s="12" t="n">
-        <v>921.11</v>
+        <v>149.06</v>
       </c>
       <c r="L32" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -1688,25 +1688,25 @@
         <v>19</v>
       </c>
       <c r="B33" s="12" t="n">
-        <v>51.25</v>
+        <v>49.76</v>
       </c>
       <c r="C33" s="12" t="n">
-        <v>102.5</v>
+        <v>49.76</v>
       </c>
       <c r="D33" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I33" s="11" t="n">
         <v>19</v>
       </c>
       <c r="J33" s="12" t="n">
-        <v>160.06</v>
+        <v>155.42</v>
       </c>
       <c r="K33" s="12" t="n">
-        <v>960.39</v>
+        <v>155.42</v>
       </c>
       <c r="L33" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -1714,25 +1714,25 @@
         <v>20</v>
       </c>
       <c r="B34" s="12" t="n">
-        <v>50.18</v>
+        <v>48.72</v>
       </c>
       <c r="C34" s="12" t="n">
-        <v>100.35</v>
+        <v>48.72</v>
       </c>
       <c r="D34" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I34" s="11" t="n">
         <v>20</v>
       </c>
       <c r="J34" s="12" t="n">
-        <v>166.89</v>
+        <v>162.05</v>
       </c>
       <c r="K34" s="12" t="n">
-        <v>1001.34</v>
+        <v>162.05</v>
       </c>
       <c r="L34" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -1740,25 +1740,25 @@
         <v>21</v>
       </c>
       <c r="B35" s="12" t="n">
-        <v>49.1</v>
+        <v>47.68</v>
       </c>
       <c r="C35" s="12" t="n">
-        <v>98.2</v>
+        <v>47.68</v>
       </c>
       <c r="D35" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I35" s="11" t="n">
         <v>21</v>
       </c>
       <c r="J35" s="12" t="n">
-        <v>174.01</v>
+        <v>168.96</v>
       </c>
       <c r="K35" s="12" t="n">
-        <v>1044.04</v>
+        <v>168.96</v>
       </c>
       <c r="L35" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -1766,25 +1766,25 @@
         <v>22</v>
       </c>
       <c r="B36" s="12" t="n">
-        <v>48.03</v>
+        <v>46.63</v>
       </c>
       <c r="C36" s="12" t="n">
-        <v>96.05</v>
+        <v>46.63</v>
       </c>
       <c r="D36" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I36" s="11" t="n">
         <v>22</v>
       </c>
       <c r="J36" s="12" t="n">
-        <v>181.43</v>
+        <v>176.16</v>
       </c>
       <c r="K36" s="12" t="n">
-        <v>1088.56</v>
+        <v>176.16</v>
       </c>
       <c r="L36" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -1792,25 +1792,25 @@
         <v>23</v>
       </c>
       <c r="B37" s="12" t="n">
-        <v>46.95</v>
+        <v>45.59</v>
       </c>
       <c r="C37" s="12" t="n">
-        <v>93.90000000000001</v>
+        <v>45.59</v>
       </c>
       <c r="D37" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I37" s="11" t="n">
         <v>23</v>
       </c>
       <c r="J37" s="12" t="n">
-        <v>189.16</v>
+        <v>183.67</v>
       </c>
       <c r="K37" s="12" t="n">
-        <v>1134.98</v>
+        <v>183.67</v>
       </c>
       <c r="L37" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -1818,25 +1818,25 @@
         <v>24</v>
       </c>
       <c r="B38" s="12" t="n">
-        <v>45.88</v>
+        <v>44.54</v>
       </c>
       <c r="C38" s="12" t="n">
-        <v>91.75</v>
+        <v>44.54</v>
       </c>
       <c r="D38" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I38" s="11" t="n">
         <v>24</v>
       </c>
       <c r="J38" s="12" t="n">
-        <v>197.23</v>
+        <v>191.51</v>
       </c>
       <c r="K38" s="12" t="n">
-        <v>1183.38</v>
+        <v>191.51</v>
       </c>
       <c r="L38" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -1844,25 +1844,25 @@
         <v>25</v>
       </c>
       <c r="B39" s="12" t="n">
-        <v>44.8</v>
+        <v>43.5</v>
       </c>
       <c r="C39" s="12" t="n">
-        <v>89.59999999999999</v>
+        <v>43.5</v>
       </c>
       <c r="D39" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I39" s="11" t="n">
         <v>25</v>
       </c>
       <c r="J39" s="12" t="n">
-        <v>205.64</v>
+        <v>199.67</v>
       </c>
       <c r="K39" s="12" t="n">
-        <v>1233.85</v>
+        <v>199.67</v>
       </c>
       <c r="L39" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -1870,25 +1870,25 @@
         <v>26</v>
       </c>
       <c r="B40" s="12" t="n">
-        <v>43.72</v>
+        <v>42.46</v>
       </c>
       <c r="C40" s="12" t="n">
-        <v>87.45</v>
+        <v>42.46</v>
       </c>
       <c r="D40" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I40" s="11" t="n">
         <v>26</v>
       </c>
       <c r="J40" s="12" t="n">
-        <v>214.41</v>
+        <v>208.19</v>
       </c>
       <c r="K40" s="12" t="n">
-        <v>1286.46</v>
+        <v>208.19</v>
       </c>
       <c r="L40" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -1896,25 +1896,25 @@
         <v>27</v>
       </c>
       <c r="B41" s="12" t="n">
-        <v>42.65</v>
+        <v>41.41</v>
       </c>
       <c r="C41" s="12" t="n">
-        <v>85.3</v>
+        <v>41.41</v>
       </c>
       <c r="D41" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I41" s="11" t="n">
         <v>27</v>
       </c>
       <c r="J41" s="12" t="n">
-        <v>223.55</v>
+        <v>217.07</v>
       </c>
       <c r="K41" s="12" t="n">
-        <v>1341.32</v>
+        <v>217.07</v>
       </c>
       <c r="L41" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -1922,25 +1922,25 @@
         <v>28</v>
       </c>
       <c r="B42" s="12" t="n">
-        <v>41.57</v>
+        <v>40.37</v>
       </c>
       <c r="C42" s="12" t="n">
-        <v>124.72</v>
+        <v>40.37</v>
       </c>
       <c r="D42" s="13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I42" s="11" t="n">
         <v>28</v>
       </c>
       <c r="J42" s="12" t="n">
-        <v>233.09</v>
+        <v>226.32</v>
       </c>
       <c r="K42" s="12" t="n">
-        <v>1398.52</v>
+        <v>226.32</v>
       </c>
       <c r="L42" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -1948,25 +1948,25 @@
         <v>29</v>
       </c>
       <c r="B43" s="12" t="n">
-        <v>40.5</v>
+        <v>39.32</v>
       </c>
       <c r="C43" s="12" t="n">
-        <v>121.5</v>
+        <v>39.32</v>
       </c>
       <c r="D43" s="13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I43" s="11" t="n">
         <v>29</v>
       </c>
       <c r="J43" s="12" t="n">
-        <v>243.03</v>
+        <v>235.97</v>
       </c>
       <c r="K43" s="12" t="n">
-        <v>1458.15</v>
+        <v>235.97</v>
       </c>
       <c r="L43" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -1974,25 +1974,25 @@
         <v>30</v>
       </c>
       <c r="B44" s="12" t="n">
-        <v>39.42</v>
+        <v>38.28</v>
       </c>
       <c r="C44" s="12" t="n">
-        <v>118.27</v>
+        <v>76.56</v>
       </c>
       <c r="D44" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I44" s="11" t="n">
         <v>30</v>
       </c>
       <c r="J44" s="12" t="n">
-        <v>253.39</v>
+        <v>246.04</v>
       </c>
       <c r="K44" s="12" t="n">
-        <v>1520.33</v>
+        <v>246.04</v>
       </c>
       <c r="L44" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update actual holdings to TQQQ 213 shares at 0.76 avg price
</commit_message>
<xml_diff>
--- a/vr_portfolio_log.xlsx
+++ b/vr_portfolio_log.xlsx
@@ -735,11 +735,11 @@
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
@@ -798,10 +798,10 @@
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="B4" s="3" t="n">
-        <v>6661.699922180176</v>
+        <v>17936.89967498779</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>3549.599922180176</v>
+        <v>14824.79967498779</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>3112.1</v>
@@ -810,14 +810,14 @@
         <v>4058.27</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>3714.058</v>
+        <v>3731.3056475</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>5024.901999999999</v>
+        <v>5048.2370525</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
     </row>
@@ -1031,19 +1031,19 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>74.08</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>51</v>
+        <v>213</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>3549.6</v>
+        <v>14824.8</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>3112.1</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>6661.7</v>
+        <v>17936.9</v>
       </c>
       <c r="H10" s="6" t="n">
         <v>4058.27</v>
@@ -1057,24 +1057,24 @@
         </is>
       </c>
       <c r="K10" s="8" t="n">
-        <v>0.0767</v>
+        <v>0.08169999999999999</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>4369.48</v>
+        <v>4389.77</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>3714.06</v>
+        <v>3731.31</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>5024.9</v>
-      </c>
-      <c r="O10" s="9" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>5048.24</v>
+      </c>
+      <c r="O10" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
         </is>
       </c>
       <c r="P10" s="6" t="n">
-        <v>819.88</v>
+        <v>10435.03</v>
       </c>
     </row>
     <row r="11">
@@ -1235,10 +1235,10 @@
         <v>73.29000000000001</v>
       </c>
       <c r="K15" s="12" t="n">
-        <v>73.29000000000001</v>
+        <v>513.0599999999999</v>
       </c>
       <c r="L15" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
@@ -1261,10 +1261,10 @@
         <v>76.42</v>
       </c>
       <c r="K16" s="12" t="n">
-        <v>76.42</v>
+        <v>534.9299999999999</v>
       </c>
       <c r="L16" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
@@ -1287,10 +1287,10 @@
         <v>79.68000000000001</v>
       </c>
       <c r="K17" s="12" t="n">
-        <v>79.68000000000001</v>
+        <v>557.74</v>
       </c>
       <c r="L17" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
@@ -1313,10 +1313,10 @@
         <v>83.08</v>
       </c>
       <c r="K18" s="12" t="n">
-        <v>83.08</v>
+        <v>581.53</v>
       </c>
       <c r="L18" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
@@ -1339,10 +1339,10 @@
         <v>86.62</v>
       </c>
       <c r="K19" s="12" t="n">
-        <v>86.62</v>
+        <v>606.33</v>
       </c>
       <c r="L19" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
@@ -1365,10 +1365,10 @@
         <v>90.31</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>90.31</v>
+        <v>632.1799999999999</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21">
@@ -1391,10 +1391,10 @@
         <v>94.16</v>
       </c>
       <c r="K21" s="12" t="n">
-        <v>94.16</v>
+        <v>659.14</v>
       </c>
       <c r="L21" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22">
@@ -1417,10 +1417,10 @@
         <v>98.18000000000001</v>
       </c>
       <c r="K22" s="12" t="n">
-        <v>98.18000000000001</v>
+        <v>687.25</v>
       </c>
       <c r="L22" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23">
@@ -1443,10 +1443,10 @@
         <v>102.36</v>
       </c>
       <c r="K23" s="12" t="n">
-        <v>102.36</v>
+        <v>716.55</v>
       </c>
       <c r="L23" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24">
@@ -1469,10 +1469,10 @@
         <v>106.73</v>
       </c>
       <c r="K24" s="12" t="n">
-        <v>106.73</v>
+        <v>747.11</v>
       </c>
       <c r="L24" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25">
@@ -1495,10 +1495,10 @@
         <v>111.28</v>
       </c>
       <c r="K25" s="12" t="n">
-        <v>111.28</v>
+        <v>778.97</v>
       </c>
       <c r="L25" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26">
@@ -1521,10 +1521,10 @@
         <v>116.03</v>
       </c>
       <c r="K26" s="12" t="n">
-        <v>116.03</v>
+        <v>812.1900000000001</v>
       </c>
       <c r="L26" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27">
@@ -1547,10 +1547,10 @@
         <v>120.97</v>
       </c>
       <c r="K27" s="12" t="n">
-        <v>120.97</v>
+        <v>846.8200000000001</v>
       </c>
       <c r="L27" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28">
@@ -1573,10 +1573,10 @@
         <v>126.13</v>
       </c>
       <c r="K28" s="12" t="n">
-        <v>126.13</v>
+        <v>882.9299999999999</v>
       </c>
       <c r="L28" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29">
@@ -1599,10 +1599,10 @@
         <v>131.51</v>
       </c>
       <c r="K29" s="12" t="n">
-        <v>131.51</v>
+        <v>920.58</v>
       </c>
       <c r="L29" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30">
@@ -1625,10 +1625,10 @@
         <v>137.12</v>
       </c>
       <c r="K30" s="12" t="n">
-        <v>137.12</v>
+        <v>959.84</v>
       </c>
       <c r="L30" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31">
@@ -1651,10 +1651,10 @@
         <v>142.97</v>
       </c>
       <c r="K31" s="12" t="n">
-        <v>142.97</v>
+        <v>1000.77</v>
       </c>
       <c r="L31" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32">
@@ -1677,10 +1677,10 @@
         <v>149.06</v>
       </c>
       <c r="K32" s="12" t="n">
-        <v>149.06</v>
+        <v>1043.44</v>
       </c>
       <c r="L32" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="33">
@@ -1703,10 +1703,10 @@
         <v>155.42</v>
       </c>
       <c r="K33" s="12" t="n">
-        <v>155.42</v>
+        <v>1087.94</v>
       </c>
       <c r="L33" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34">
@@ -1729,10 +1729,10 @@
         <v>162.05</v>
       </c>
       <c r="K34" s="12" t="n">
-        <v>162.05</v>
+        <v>1134.33</v>
       </c>
       <c r="L34" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35">
@@ -1755,10 +1755,10 @@
         <v>168.96</v>
       </c>
       <c r="K35" s="12" t="n">
-        <v>168.96</v>
+        <v>1182.7</v>
       </c>
       <c r="L35" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36">
@@ -1781,10 +1781,10 @@
         <v>176.16</v>
       </c>
       <c r="K36" s="12" t="n">
-        <v>176.16</v>
+        <v>1233.14</v>
       </c>
       <c r="L36" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37">
@@ -1807,10 +1807,10 @@
         <v>183.67</v>
       </c>
       <c r="K37" s="12" t="n">
-        <v>183.67</v>
+        <v>1285.72</v>
       </c>
       <c r="L37" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38">
@@ -1833,10 +1833,10 @@
         <v>191.51</v>
       </c>
       <c r="K38" s="12" t="n">
-        <v>191.51</v>
+        <v>1340.55</v>
       </c>
       <c r="L38" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39">
@@ -1859,10 +1859,10 @@
         <v>199.67</v>
       </c>
       <c r="K39" s="12" t="n">
-        <v>199.67</v>
+        <v>1397.72</v>
       </c>
       <c r="L39" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40">
@@ -1885,10 +1885,10 @@
         <v>208.19</v>
       </c>
       <c r="K40" s="12" t="n">
-        <v>208.19</v>
+        <v>1457.32</v>
       </c>
       <c r="L40" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="41">
@@ -1911,10 +1911,10 @@
         <v>217.07</v>
       </c>
       <c r="K41" s="12" t="n">
-        <v>217.07</v>
+        <v>1519.46</v>
       </c>
       <c r="L41" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="42">
@@ -1937,10 +1937,10 @@
         <v>226.32</v>
       </c>
       <c r="K42" s="12" t="n">
-        <v>226.32</v>
+        <v>1584.26</v>
       </c>
       <c r="L42" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43">
@@ -1963,10 +1963,10 @@
         <v>235.97</v>
       </c>
       <c r="K43" s="12" t="n">
-        <v>235.97</v>
+        <v>1651.81</v>
       </c>
       <c r="L43" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44">
@@ -1989,10 +1989,10 @@
         <v>246.04</v>
       </c>
       <c r="K44" s="12" t="n">
-        <v>246.04</v>
+        <v>1722.25</v>
       </c>
       <c r="L44" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor holdings fallback to dynamically read variables from vr_state.json without hardcoded constants
</commit_message>
<xml_diff>
--- a/vr_portfolio_log.xlsx
+++ b/vr_portfolio_log.xlsx
@@ -738,8 +738,8 @@
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
@@ -807,13 +807,13 @@
         <v>3112.1</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>4058.27</v>
+        <v>4389.77135</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>3731.3056475</v>
+        <v>4014.4906757375</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>5048.2370525</v>
+        <v>5431.369737762499</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
@@ -1046,10 +1046,10 @@
         <v>17936.9</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>4058.27</v>
+        <v>4389.77</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>0.7669</v>
+        <v>0.7089</v>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
@@ -1057,16 +1057,16 @@
         </is>
       </c>
       <c r="K10" s="8" t="n">
-        <v>0.08169999999999999</v>
+        <v>0.0759</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>4389.77</v>
+        <v>4722.93</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>3731.31</v>
+        <v>4014.49</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>5048.24</v>
+        <v>5431.37</v>
       </c>
       <c r="O10" s="18" t="inlineStr">
         <is>
@@ -1074,7 +1074,7 @@
         </is>
       </c>
       <c r="P10" s="6" t="n">
-        <v>10435.03</v>
+        <v>10101.87</v>
       </c>
     </row>
     <row r="11">

</xml_diff>